<commit_message>
Update band review files for 2018–2024
- 2018: manual corrections to banded bird entries (band combos clarified,
  numbering fixed) after biologist review of the structured band cells
- 2019–2024: regenerated band review files using updated parse_bands.py
  (count-first philosophy: every cell numbered even if notation is unclear;
  pink flag reserved only for cases where bird count is genuinely unknown)

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Databases/Database3BandReview/Winter Birds 2018 Band Review.xlsx
+++ b/Databases/Database3BandReview/Winter Birds 2018 Band Review.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rohanpoudel/Documents/USFWS/PipingPlover/Databases/Database3BandReview/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5521CF1E-86CD-4041-8268-B6ADE615F193}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C7D7322-2070-5B42-9F8E-E2C9B34D2FED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4220" yWindow="-21000" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19820" yWindow="-28200" windowWidth="34400" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="259">
   <si>
     <t>Transect</t>
   </si>
@@ -812,16 +812,7 @@
     <t>Disappointed that we saw no Red Knots. Surprised by the first ever American Avocets I've ever seen at the ocean shoreline.</t>
   </si>
   <si>
-    <t>4 Unbanded, 1) Banded - FK[UN], _ : S, _</t>
-  </si>
-  <si>
     <t>1) S/LY:bf/LG (bf = light blue flag, no code); reported directly to bander</t>
-  </si>
-  <si>
-    <t>0 banded birds then none readable</t>
-  </si>
-  <si>
-    <t>this is just one says here. One individual. Band/flag code:1) YX6, color: green, position: upper left". The "O" is for an orange band on the right leg, position: upper right.</t>
   </si>
   <si>
     <t>1) Left leg: Orange flag, upper yellow band, lower green band. Right leg: Upper silver USFWS band, lower Yellow band</t>
@@ -843,6 +834,12 @@
   </si>
   <si>
     <t>1)S, K : FO, B/Y FTP; Y; FTP, - : -, - reported to Great Lakes area researchers</t>
+  </si>
+  <si>
+    <t>1) YX6, color: green, position: upper left". The "O" is for an orange band on the right leg, position: upper right.</t>
+  </si>
+  <si>
+    <t>1) Banded - FK[UN], _ : S, _</t>
   </si>
 </sst>
 </file>
@@ -2058,9 +2055,7 @@
       <c r="R8">
         <v>17</v>
       </c>
-      <c r="S8" s="2" t="s">
-        <v>252</v>
-      </c>
+      <c r="S8" s="2"/>
       <c r="T8">
         <v>30.506930000000001</v>
       </c>
@@ -2626,7 +2621,7 @@
         <v>1</v>
       </c>
       <c r="BC14" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="BD14">
         <v>30.329180000000001</v>
@@ -2694,7 +2689,7 @@
         <v>9</v>
       </c>
       <c r="S15" s="2" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="T15">
         <v>25.489989999999999</v>
@@ -3222,7 +3217,7 @@
         <v>5</v>
       </c>
       <c r="AI21" s="2" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="AJ21">
         <v>30.4329</v>
@@ -3349,7 +3344,7 @@
         <v>2</v>
       </c>
       <c r="S23" s="2" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
     </row>
     <row r="24" spans="1:83" ht="128" x14ac:dyDescent="0.2">
@@ -3405,7 +3400,7 @@
         <v>8</v>
       </c>
       <c r="S24" s="3" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="25" spans="1:83" x14ac:dyDescent="0.2">
@@ -3461,7 +3456,7 @@
         <v>1</v>
       </c>
       <c r="W25" s="2" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
     </row>
     <row r="26" spans="1:83" x14ac:dyDescent="0.2">
@@ -3582,7 +3577,7 @@
         <v>10</v>
       </c>
       <c r="W27" s="2" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="28" spans="1:83" x14ac:dyDescent="0.2">
@@ -3647,7 +3642,7 @@
         <v>2</v>
       </c>
       <c r="W28" s="2" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="X28">
         <v>27.650099999999998</v>
@@ -3659,7 +3654,7 @@
         <v>15</v>
       </c>
       <c r="AA28" s="2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
     </row>
     <row r="29" spans="1:83" x14ac:dyDescent="0.2">

</xml_diff>